<commit_message>
feat(tool): Add Label Integration (Update convert_library_v2.py) (#2891)
* Add Label Support

- Added label parsing logic
- [tools] README.md: Added "labels" field description
- Added "labels" field example in "example_framework.xlsx"

* Fix typo in README.md

* Fix for CodeFactor

* Fix Typos & Update Label Verification

* Merge branch 'main' into CA-1392-Add-Label-integration-to-convert_library_v2.py

* Make code more pythonic

* avoid duplicate / fix NIS2 lib

* Update README.md

---------

Co-authored-by: eric-intuitem <71850047+eric-intuitem@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tools/example_framework.xlsx
+++ b/tools/example_framework.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\tarkadia\projects\intuitem\ciso-assistant-community\tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E84F6D-1951-4647-B96B-120B76A95CF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D1C6024-1613-47E4-AAEF-428390C867CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1485" yWindow="-15870" windowWidth="25440" windowHeight="15990" tabRatio="907" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -77,7 +77,32 @@
         </r>
       </text>
     </comment>
-    <comment ref="A11" authorId="0" shapeId="0" xr:uid="{8377CD80-173C-4910-ABAF-16B301C42544}">
+    <comment ref="A11" authorId="0" shapeId="0" xr:uid="{FCDB3F77-8B06-4998-BCDC-B60DCE09EC36}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">.: About label :.
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Works like the hashtag system in social media. Labels mustn't contains spaces. They are  separated by line breaks or commas.
+All labels will be forced to uppercase in the resulting YAML file.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A12" authorId="0" shapeId="0" xr:uid="{8377CD80-173C-4910-ABAF-16B301C42544}">
       <text>
         <r>
           <rPr>
@@ -666,7 +691,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="553">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="555">
   <si>
     <t>type</t>
   </si>
@@ -2541,12 +2566,18 @@
   <si>
     <t>nice_to_have</t>
   </si>
+  <si>
+    <t>labels</t>
+  </si>
+  <si>
+    <t>example_framework, framework1, my-very-cool-framework, I-LOVE-MY-FRAMEWORK</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2719,6 +2750,13 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="18">
@@ -3255,6 +3293,24 @@
     <xf numFmtId="0" fontId="13" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3308,24 +3364,6 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4820,55 +4858,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="62.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="112" t="s">
+      <c r="A1" s="94" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
-      <c r="H1" s="113"/>
-      <c r="I1" s="113"/>
-      <c r="J1" s="113"/>
-      <c r="K1" s="113"/>
-      <c r="L1" s="113"/>
-      <c r="M1" s="114"/>
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="95"/>
+      <c r="I1" s="95"/>
+      <c r="J1" s="95"/>
+      <c r="K1" s="95"/>
+      <c r="L1" s="95"/>
+      <c r="M1" s="96"/>
     </row>
     <row r="2" spans="1:13" ht="42.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="115" t="s">
+      <c r="A2" s="97" t="s">
         <v>544</v>
       </c>
-      <c r="B2" s="116"/>
-      <c r="C2" s="116"/>
-      <c r="D2" s="116"/>
-      <c r="E2" s="116"/>
-      <c r="F2" s="116"/>
-      <c r="G2" s="116"/>
-      <c r="H2" s="116"/>
-      <c r="I2" s="116"/>
-      <c r="J2" s="116"/>
-      <c r="K2" s="116"/>
-      <c r="L2" s="116"/>
-      <c r="M2" s="117"/>
+      <c r="B2" s="98"/>
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
+      <c r="I2" s="98"/>
+      <c r="J2" s="98"/>
+      <c r="K2" s="98"/>
+      <c r="L2" s="98"/>
+      <c r="M2" s="99"/>
     </row>
     <row r="3" spans="1:13" ht="34.799999999999997" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="94" t="s">
+      <c r="A3" s="100" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="95"/>
-      <c r="C3" s="95"/>
-      <c r="D3" s="95"/>
-      <c r="E3" s="95"/>
-      <c r="F3" s="95"/>
-      <c r="G3" s="95"/>
-      <c r="H3" s="95"/>
-      <c r="I3" s="95"/>
-      <c r="J3" s="95"/>
-      <c r="K3" s="95"/>
-      <c r="L3" s="95"/>
-      <c r="M3" s="96"/>
+      <c r="B3" s="101"/>
+      <c r="C3" s="101"/>
+      <c r="D3" s="101"/>
+      <c r="E3" s="101"/>
+      <c r="F3" s="101"/>
+      <c r="G3" s="101"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="101"/>
+      <c r="J3" s="101"/>
+      <c r="K3" s="101"/>
+      <c r="L3" s="101"/>
+      <c r="M3" s="102"/>
     </row>
     <row r="4" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="85" t="s">
@@ -5042,50 +5080,50 @@
       <c r="M12" s="81"/>
     </row>
     <row r="13" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="97" t="s">
+      <c r="A13" s="103" t="s">
         <v>42</v>
       </c>
-      <c r="B13" s="97"/>
-      <c r="C13" s="98" t="s">
+      <c r="B13" s="103"/>
+      <c r="C13" s="104" t="s">
         <v>543</v>
       </c>
-      <c r="D13" s="99"/>
-      <c r="E13" s="99"/>
-      <c r="F13" s="99"/>
-      <c r="G13" s="99"/>
-      <c r="H13" s="99"/>
-      <c r="I13" s="99"/>
-      <c r="J13" s="99"/>
-      <c r="K13" s="99"/>
-      <c r="L13" s="99"/>
-      <c r="M13" s="99"/>
+      <c r="D13" s="105"/>
+      <c r="E13" s="105"/>
+      <c r="F13" s="105"/>
+      <c r="G13" s="105"/>
+      <c r="H13" s="105"/>
+      <c r="I13" s="105"/>
+      <c r="J13" s="105"/>
+      <c r="K13" s="105"/>
+      <c r="L13" s="105"/>
+      <c r="M13" s="105"/>
     </row>
     <row r="14" spans="1:13" ht="34.799999999999997" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="94" t="s">
+      <c r="A14" s="100" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="95"/>
-      <c r="C14" s="95"/>
-      <c r="D14" s="95"/>
-      <c r="E14" s="95"/>
-      <c r="F14" s="95"/>
-      <c r="G14" s="95"/>
-      <c r="H14" s="95"/>
-      <c r="I14" s="95"/>
-      <c r="J14" s="95"/>
-      <c r="K14" s="95"/>
-      <c r="L14" s="95"/>
-      <c r="M14" s="96"/>
+      <c r="B14" s="101"/>
+      <c r="C14" s="101"/>
+      <c r="D14" s="101"/>
+      <c r="E14" s="101"/>
+      <c r="F14" s="101"/>
+      <c r="G14" s="101"/>
+      <c r="H14" s="101"/>
+      <c r="I14" s="101"/>
+      <c r="J14" s="101"/>
+      <c r="K14" s="101"/>
+      <c r="L14" s="101"/>
+      <c r="M14" s="102"/>
     </row>
     <row r="15" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="109" t="s">
+      <c r="A15" s="115" t="s">
         <v>258</v>
       </c>
-      <c r="B15" s="110"/>
-      <c r="C15" s="110"/>
-      <c r="D15" s="110"/>
-      <c r="E15" s="110"/>
-      <c r="F15" s="111"/>
+      <c r="B15" s="116"/>
+      <c r="C15" s="116"/>
+      <c r="D15" s="116"/>
+      <c r="E15" s="116"/>
+      <c r="F15" s="117"/>
       <c r="G15" s="79" t="s">
         <v>263</v>
       </c>
@@ -5116,14 +5154,14 @@
       <c r="M16" s="81"/>
     </row>
     <row r="17" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="106" t="s">
+      <c r="A17" s="112" t="s">
         <v>48</v>
       </c>
-      <c r="B17" s="107"/>
-      <c r="C17" s="107"/>
-      <c r="D17" s="107"/>
-      <c r="E17" s="107"/>
-      <c r="F17" s="108"/>
+      <c r="B17" s="113"/>
+      <c r="C17" s="113"/>
+      <c r="D17" s="113"/>
+      <c r="E17" s="113"/>
+      <c r="F17" s="114"/>
       <c r="G17" s="79" t="s">
         <v>260</v>
       </c>
@@ -5135,14 +5173,14 @@
       <c r="M17" s="81"/>
     </row>
     <row r="18" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="103" t="s">
+      <c r="A18" s="109" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="104"/>
-      <c r="C18" s="104"/>
-      <c r="D18" s="104"/>
-      <c r="E18" s="104"/>
-      <c r="F18" s="105"/>
+      <c r="B18" s="110"/>
+      <c r="C18" s="110"/>
+      <c r="D18" s="110"/>
+      <c r="E18" s="110"/>
+      <c r="F18" s="111"/>
       <c r="G18" s="79" t="s">
         <v>261</v>
       </c>
@@ -5154,14 +5192,14 @@
       <c r="M18" s="81"/>
     </row>
     <row r="19" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="100" t="s">
+      <c r="A19" s="106" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="101"/>
-      <c r="C19" s="101"/>
-      <c r="D19" s="101"/>
-      <c r="E19" s="101"/>
-      <c r="F19" s="102"/>
+      <c r="B19" s="107"/>
+      <c r="C19" s="107"/>
+      <c r="D19" s="107"/>
+      <c r="E19" s="107"/>
+      <c r="F19" s="108"/>
       <c r="G19" s="79" t="s">
         <v>47</v>
       </c>
@@ -5173,23 +5211,23 @@
       <c r="M19" s="81"/>
     </row>
     <row r="20" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="97" t="s">
+      <c r="A20" s="103" t="s">
         <v>49</v>
       </c>
-      <c r="B20" s="97"/>
-      <c r="C20" s="98" t="s">
+      <c r="B20" s="103"/>
+      <c r="C20" s="104" t="s">
         <v>262</v>
       </c>
-      <c r="D20" s="99"/>
-      <c r="E20" s="99"/>
-      <c r="F20" s="99"/>
-      <c r="G20" s="99"/>
-      <c r="H20" s="99"/>
-      <c r="I20" s="99"/>
-      <c r="J20" s="99"/>
-      <c r="K20" s="99"/>
-      <c r="L20" s="99"/>
-      <c r="M20" s="99"/>
+      <c r="D20" s="105"/>
+      <c r="E20" s="105"/>
+      <c r="F20" s="105"/>
+      <c r="G20" s="105"/>
+      <c r="H20" s="105"/>
+      <c r="I20" s="105"/>
+      <c r="J20" s="105"/>
+      <c r="K20" s="105"/>
+      <c r="L20" s="105"/>
+      <c r="M20" s="105"/>
     </row>
     <row r="21" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
@@ -6824,7 +6862,7 @@
   <sheetPr codeName="Feuil2">
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
@@ -6913,33 +6951,41 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="78" t="s">
+        <v>553</v>
+      </c>
+      <c r="B11" s="36" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="78" t="s">
         <v>535</v>
       </c>
-      <c r="B11" s="31" t="s">
+      <c r="B12" s="31" t="s">
         <v>536</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="36" t="s">
+      <c r="B13" s="36" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="8" t="s">
+    <row r="14" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="37" t="s">
+      <c r="B14" s="37" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" s="8" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="36" t="s">
+      <c r="B15" s="36" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>